<commit_message>
Checkpoint: Shipping/Field board parity, locked dashboard statuses, and Trade/Material column repair.
Align ghost boards with dashboard visibility, keep spooling/fab/shipping/field statuses dashboard-driven, restore Trade/Material section sync, and clean up SSv3 weld-log PDF entry fields.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Spooling Savant Version 3 (Exports)/Boardroom/Exports/Piping Specification Catalog.xlsx
+++ b/Spooling Savant Version 3 (Exports)/Boardroom/Exports/Piping Specification Catalog.xlsx
@@ -121,7 +121,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>EL90-CS-CARBONSTEEL-6</t>
+          <t>EL90-CS-CARBONSTEEL-3</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -131,22 +131,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>6 in</t>
+          <t>3 in</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>6.625 in</t>
+          <t>3.500 in</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0.283 in</t>
+          <t>0.216 in</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>6.060 in</t>
+          <t>3.068 in</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -168,12 +168,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>FLG-CS-CARBONSTEEL-6</t>
+          <t>EL90-CS-CARBONSTEEL-6</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Flange</t>
+          <t>Elbow</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -188,12 +188,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0.280 in</t>
+          <t>0.283 in</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>6.065 in</t>
+          <t>6.060 in</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -215,32 +215,32 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>OLET-CS-FORGEDSTEEL-6</t>
+          <t>FLG-CS-CARBONSTEEL-3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Olet</t>
+          <t>Flange</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>6 in</t>
+          <t>3 in</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6.000 in</t>
+          <t>3.500 in</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t/>
+          <t>0.216 in</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>6.000 in</t>
+          <t>3.068 in</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -250,7 +250,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Forged Steel</t>
+          <t>Carbon Steel</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -262,12 +262,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PIPE-CS-CARBONSTEEL-6</t>
+          <t>FLG-CS-CARBONSTEEL-6</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Pipe</t>
+          <t>Flange</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -309,45 +309,233 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>OLET-CS-CARBONSTEEL-3</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Olet</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>3 in</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>3.500 in</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0.216 in</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>3.068 in</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Carbon Steel</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Steel</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>OLET-CS-FORGEDSTEEL-6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Olet</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>6 in</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>6.000 in</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>6.000 in</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Forged Steel</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Steel</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>PIPE-CS-CARBONSTEEL-3</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Pipe</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>3 in</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>3.500 in</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0.216 in</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>3.068 in</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Carbon Steel</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Steel</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>PIPE-CS-CARBONSTEEL-6</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Pipe</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>6 in</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>6.625 in</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>0.280 in</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>6.065 in</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Carbon Steel</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Steel</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>TEE-CS-CARBONSTEEL-6</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Tee</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>6 in</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>6.625 in</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>0.283 in</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>6.060 in</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Carbon Steel</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
+      <c r="G10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Carbon Steel</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
         <is>
           <t>Steel</t>
         </is>

</xml_diff>

<commit_message>
Checkpoint: fab shop worker flow, Detailers origin mirror, and Main Overview Fab sections.
Shop workers get limited nav with queue view-only access; owners see worker stations. Keep Detailers origin visibility through Fab, fix due-date edits, and show Fab packages on Main Overview.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Spooling Savant Version 3 (Exports)/Boardroom/Exports/Piping Specification Catalog.xlsx
+++ b/Spooling Savant Version 3 (Exports)/Boardroom/Exports/Piping Specification Catalog.xlsx
@@ -121,7 +121,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>EL90-CS-CARBONSTEEL-3</t>
+          <t>EL45-CS-CARBONSTEEL-3</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -168,7 +168,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>EL90-CS-CARBONSTEEL-6</t>
+          <t>EL90-CS-CARBONSTEEL-3</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -178,22 +178,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>6 in</t>
+          <t>3 in</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>6.625 in</t>
+          <t>3.500 in</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0.283 in</t>
+          <t>0.216 in</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>6.060 in</t>
+          <t>3.068 in</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -215,32 +215,32 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>FLG-CS-CARBONSTEEL-3</t>
+          <t>EL90-CS-CARBONSTEEL-6</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Flange</t>
+          <t>Elbow</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3 in</t>
+          <t>6 in</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3.500 in</t>
+          <t>6.625 in</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0.216 in</t>
+          <t>0.283 in</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3.068 in</t>
+          <t>6.060 in</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -262,7 +262,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>FLG-CS-CARBONSTEEL-6</t>
+          <t>FLG-CS-CARBONSTEEL-2P5</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -272,22 +272,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6 in</t>
+          <t>2.5 in</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.625 in</t>
+          <t>2.875 in</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0.280 in</t>
+          <t>0.201 in</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>6.065 in</t>
+          <t>2.474 in</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -309,12 +309,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>OLET-CS-CARBONSTEEL-3</t>
+          <t>FLG-CS-CARBONSTEEL-3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Olet</t>
+          <t>Flange</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -356,12 +356,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>OLET-CS-FORGEDSTEEL-6</t>
+          <t>FLG-CS-CARBONSTEEL-6</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Olet</t>
+          <t>Flange</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -371,17 +371,17 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>6.000 in</t>
+          <t>6.625 in</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t/>
+          <t>0.280 in</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6.000 in</t>
+          <t>6.065 in</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -391,7 +391,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Forged Steel</t>
+          <t>Carbon Steel</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -403,12 +403,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PIPE-CS-CARBONSTEEL-3</t>
+          <t>OLET-CS-CARBONSTEEL-3</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Pipe</t>
+          <t>Olet</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -450,12 +450,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PIPE-CS-CARBONSTEEL-6</t>
+          <t>OLET-CS-FORGEDSTEEL-6</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Pipe</t>
+          <t>Olet</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -465,17 +465,17 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>6.625 in</t>
+          <t>6.000 in</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.280 in</t>
+          <t/>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>6.065 in</t>
+          <t>6.000 in</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -485,7 +485,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Carbon Steel</t>
+          <t>Forged Steel</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -497,45 +497,186 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>PIPE-CS-CARBONSTEEL-3</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Pipe</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>3 in</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>3.500 in</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>0.216 in</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>3.068 in</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Carbon Steel</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Steel</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>PIPE-CS-CARBONSTEEL-6</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Pipe</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>6 in</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>6.625 in</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>0.280 in</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>6.065 in</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Carbon Steel</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Steel</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>RED-CS-CARBONSTEEL-3</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Reducer</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>3 in</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>3.500 in</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>0.216 in</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>3.068 in</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Carbon Steel</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Steel</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>TEE-CS-CARBONSTEEL-6</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Tee</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>6 in</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>6.625 in</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>0.283 in</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>6.060 in</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Carbon Steel</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
+      <c r="G13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Carbon Steel</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
         <is>
           <t>Steel</t>
         </is>

</xml_diff>